<commit_message>
Revert "Merge branch 'develop' into codex"
This reverts commit 773b7e6f783ddca6367b0ae02961ed2a187a9863, reversing
changes made to 12ed3e5cffb0ce20ae50f0bf8833495d7a8b5836.
</commit_message>
<xml_diff>
--- a/document/TaskMan_タスク一覧画面_ユースケース.xlsx
+++ b/document/TaskMan_タスク一覧画面_ユースケース.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\TaskMan\document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER112\Desktop\プロジェクト演習\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29E86BD-EF0B-4B43-A647-E2FD633FB5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F01074DA-340A-4F0C-9E99-479F8BF69C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2850" yWindow="1515" windowWidth="15225" windowHeight="8190" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="表紙" sheetId="1" r:id="rId1"/>
@@ -257,6 +257,19 @@
     <phoneticPr fontId="8"/>
   </si>
   <si>
+    <t>登録されているタスク一覧を表示する</t>
+    <rPh sb="0" eb="2">
+      <t>トウロク</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>イチラン</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ヒョウジ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
     <t>従業員</t>
     <rPh sb="0" eb="3">
       <t>ジュウギョウイン</t>
@@ -270,6 +283,46 @@
     </rPh>
     <rPh sb="8" eb="9">
       <t>ズ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>1.従業員がメニュー画面を表示する。
+2.従業員が「タスク一覧」を選択する。
+3.システムがデータベースからタスク情報を取得する。
+4.システムがタスク一覧画面を表示する。</t>
+    <rPh sb="2" eb="5">
+      <t>ジュウギョウイン</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ガメン</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ヒョウジ</t>
+    </rPh>
+    <rPh sb="21" eb="24">
+      <t>ジュウギョウイン</t>
+    </rPh>
+    <rPh sb="29" eb="31">
+      <t>イチラン</t>
+    </rPh>
+    <rPh sb="33" eb="35">
+      <t>センタク</t>
+    </rPh>
+    <rPh sb="57" eb="59">
+      <t>ジョウホウ</t>
+    </rPh>
+    <rPh sb="60" eb="62">
+      <t>シュトク</t>
+    </rPh>
+    <rPh sb="76" eb="78">
+      <t>イチラン</t>
+    </rPh>
+    <rPh sb="78" eb="80">
+      <t>ガメン</t>
+    </rPh>
+    <rPh sb="81" eb="83">
+      <t>ヒョウジ</t>
     </rPh>
     <phoneticPr fontId="8"/>
   </si>
@@ -288,57 +341,34 @@
     <phoneticPr fontId="8"/>
   </si>
   <si>
-    <t>登録済みのタスク一覧を表示し、対象タスクを選択して編集画面または削除画面へ遷移する</t>
-    <rPh sb="0" eb="2">
-      <t>トウロク</t>
+    <t>E1:タスク情報が存在しない場合
+E1-1:「表示するタスクがありません」を表示
+E2.システムエラーが発生した場合
+E2-1.システムがエラーメッセージを表示</t>
+    <rPh sb="6" eb="8">
+      <t>ジョウホウ</t>
     </rPh>
-    <rPh sb="2" eb="3">
-      <t>ズ</t>
+    <rPh sb="9" eb="11">
+      <t>ソンザイ</t>
     </rPh>
-    <rPh sb="8" eb="10">
-      <t>イチラン</t>
+    <rPh sb="14" eb="16">
+      <t>バアイ</t>
     </rPh>
-    <rPh sb="11" eb="13">
+    <rPh sb="23" eb="25">
       <t>ヒョウジ</t>
     </rPh>
-    <rPh sb="15" eb="17">
-      <t>タイショウ</t>
+    <rPh sb="38" eb="40">
+      <t>ヒョウジ</t>
     </rPh>
-    <rPh sb="21" eb="23">
-      <t>センタク</t>
+    <rPh sb="53" eb="55">
+      <t>ハッセイ</t>
     </rPh>
-    <rPh sb="25" eb="27">
-      <t>ヘンシュウ</t>
+    <rPh sb="57" eb="59">
+      <t>バアイ</t>
     </rPh>
-    <rPh sb="32" eb="34">
-      <t>サクジョ</t>
+    <rPh sb="79" eb="81">
+      <t>ヒョウジ</t>
     </rPh>
-    <rPh sb="34" eb="36">
-      <t>ガメン</t>
-    </rPh>
-    <rPh sb="37" eb="39">
-      <t>センイ</t>
-    </rPh>
-    <phoneticPr fontId="8"/>
-  </si>
-  <si>
-    <t>1.利用者がメニュー画面で「タスク一覧」を選択する
-2.システムがタスク情報を取得する
-3.システムがタスク一覧画面を表示する
-4.利用者がラジオボタンで対象タスクを1件選択する
-5.利用者が「編集」または「削除」ボタンを押下する
-6.システムが選択されたタスクIDを取得する
-7.編集の場合、タスク編集画面へ遷移する
-8.削除の場合、タスク削除確認画面へ遷移する</t>
-    <phoneticPr fontId="8"/>
-  </si>
-  <si>
-    <t xml:space="preserve">E1:タスクが存在しない
-E1-1:「表示するタスクがありません。」を表示する   
-E1-2:未選択で編集ボタン押下  「対象のタスクを選択してください。」を表示する 
-E1-3:未選択で削除ボタン押下  「対象のタスクを選択してください。」を表示する 
-E2:システムエラー
-E2-1:「システムエラーが発生しました。」を表示する  </t>
     <phoneticPr fontId="8"/>
   </si>
 </sst>
@@ -367,7 +397,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1206,206 +1235,206 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="56" fontId="5" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="56" fontId="5" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1631,85 +1660,85 @@
   <sheetData>
     <row r="1" spans="3:16" ht="30" customHeight="1"/>
     <row r="2" spans="3:16" ht="30" customHeight="1">
-      <c r="C2" s="81" t="s">
+      <c r="C2" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="82"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="77"/>
       <c r="P2" s="1"/>
     </row>
     <row r="3" spans="3:16" ht="30" customHeight="1">
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
-      <c r="L3" s="54"/>
-      <c r="M3" s="54"/>
-      <c r="N3" s="54"/>
-      <c r="O3" s="54"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
       <c r="P3" s="1"/>
     </row>
     <row r="4" spans="3:16" ht="30" customHeight="1">
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="54"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="59"/>
       <c r="P4" s="1"/>
     </row>
     <row r="5" spans="3:16" ht="30" customHeight="1">
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="54"/>
-      <c r="O5" s="54"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="59"/>
+      <c r="L5" s="59"/>
+      <c r="M5" s="59"/>
+      <c r="N5" s="59"/>
+      <c r="O5" s="59"/>
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="3:16" ht="30" customHeight="1">
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="54"/>
-      <c r="N6" s="54"/>
-      <c r="O6" s="54"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59"/>
+      <c r="J6" s="59"/>
+      <c r="K6" s="59"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="59"/>
+      <c r="N6" s="59"/>
+      <c r="O6" s="59"/>
       <c r="P6" s="1"/>
     </row>
     <row r="7" spans="3:16" ht="30" customHeight="1">
@@ -1729,46 +1758,46 @@
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="3:16" ht="30" customHeight="1">
-      <c r="E8" s="83" t="s">
+      <c r="E8" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="54"/>
-      <c r="K8" s="54"/>
-      <c r="L8" s="54"/>
-      <c r="M8" s="54"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
     </row>
     <row r="9" spans="3:16" ht="30" customHeight="1"/>
     <row r="10" spans="3:16" ht="30" customHeight="1"/>
     <row r="11" spans="3:16" ht="30" customHeight="1"/>
     <row r="12" spans="3:16" ht="30" customHeight="1"/>
     <row r="13" spans="3:16" ht="15.75" customHeight="1">
-      <c r="G13" s="79" t="s">
+      <c r="G13" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="H13" s="62"/>
-      <c r="I13" s="79" t="s">
+      <c r="H13" s="49"/>
+      <c r="I13" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="J13" s="45"/>
-      <c r="K13" s="62"/>
+      <c r="J13" s="48"/>
+      <c r="K13" s="49"/>
     </row>
     <row r="14" spans="3:16" ht="15.75" customHeight="1">
-      <c r="G14" s="79"/>
-      <c r="H14" s="62"/>
-      <c r="I14" s="79"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="62"/>
+      <c r="G14" s="74"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="74"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="49"/>
     </row>
     <row r="15" spans="3:16" ht="15.75" customHeight="1">
-      <c r="G15" s="79"/>
-      <c r="H15" s="62"/>
-      <c r="I15" s="79"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="62"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="74"/>
+      <c r="J15" s="48"/>
+      <c r="K15" s="49"/>
     </row>
     <row r="16" spans="3:16" ht="15.75" customHeight="1">
       <c r="G16" s="3"/>
@@ -1777,13 +1806,13 @@
       <c r="J16" s="3"/>
     </row>
     <row r="17" spans="7:11" ht="30" customHeight="1">
-      <c r="G17" s="80" t="s">
+      <c r="G17" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="H17" s="54"/>
-      <c r="I17" s="54"/>
-      <c r="J17" s="54"/>
-      <c r="K17" s="54"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="59"/>
     </row>
     <row r="18" spans="7:11" ht="14.25" customHeight="1"/>
     <row r="19" spans="7:11" ht="24.75" customHeight="1"/>
@@ -2797,19 +2826,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="86" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="73" t="s">
+      <c r="B1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="73" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="60"/>
+      <c r="G1" s="67"/>
       <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
@@ -2821,192 +2850,192 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="74" t="s">
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="75"/>
-      <c r="F2" s="74" t="s">
+      <c r="E2" s="39"/>
+      <c r="F2" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="G2" s="75"/>
-      <c r="H2" s="78">
+      <c r="G2" s="39"/>
+      <c r="H2" s="42">
         <v>46176</v>
       </c>
-      <c r="I2" s="67" t="s">
+      <c r="I2" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="J2" s="70"/>
+      <c r="J2" s="45"/>
     </row>
     <row r="3" spans="1:10" ht="18" customHeight="1">
-      <c r="A3" s="53"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="71"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="18" customHeight="1">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="77"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
-      <c r="J4" s="72"/>
+      <c r="A4" s="87"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="80"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="82"/>
     </row>
     <row r="5" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A5" s="59" t="s">
+      <c r="A5" s="89" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="60"/>
-      <c r="D5" s="41" t="s">
+      <c r="B5" s="52"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="93" t="s">
         <v>70</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="43"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="84" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="44" t="s">
+      <c r="B6" s="48"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="61" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="54"/>
+    </row>
+    <row r="7" spans="1:10" ht="26.25" customHeight="1">
+      <c r="A7" s="84" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="48"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="61" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="54"/>
+    </row>
+    <row r="8" spans="1:10" ht="26.25" customHeight="1">
+      <c r="A8" s="84" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="48"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="61" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="54"/>
+    </row>
+    <row r="9" spans="1:10" ht="64.5" customHeight="1">
+      <c r="A9" s="90" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="83" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="49"/>
+      <c r="D9" s="104" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="54"/>
+    </row>
+    <row r="10" spans="1:10" ht="64.5" customHeight="1">
+      <c r="A10" s="91"/>
+      <c r="B10" s="83" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="49"/>
+      <c r="D10" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="46"/>
-    </row>
-    <row r="7" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A7" s="61" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="46"/>
-    </row>
-    <row r="8" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A8" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="46"/>
-    </row>
-    <row r="9" spans="1:10" ht="140.25" customHeight="1">
-      <c r="A9" s="63" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="66" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="62"/>
-      <c r="D9" s="47" t="s">
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="54"/>
+    </row>
+    <row r="11" spans="1:10" ht="99.75" customHeight="1">
+      <c r="A11" s="92"/>
+      <c r="B11" s="83" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="49"/>
+      <c r="D11" s="104" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="54"/>
+    </row>
+    <row r="12" spans="1:10" ht="99.75" customHeight="1">
+      <c r="A12" s="84" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="48"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="46"/>
-    </row>
-    <row r="10" spans="1:10" ht="64.5" customHeight="1">
-      <c r="A10" s="64"/>
-      <c r="B10" s="66" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="62"/>
-      <c r="D10" s="44" t="s">
-        <v>73</v>
-      </c>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="46"/>
-    </row>
-    <row r="11" spans="1:10" ht="99.75" customHeight="1">
-      <c r="A11" s="65"/>
-      <c r="B11" s="66" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="62"/>
-      <c r="D11" s="47" t="s">
-        <v>77</v>
-      </c>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="46"/>
-    </row>
-    <row r="12" spans="1:10" ht="99.75" customHeight="1">
-      <c r="A12" s="61" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="44" t="s">
-        <v>74</v>
-      </c>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="46"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="48"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="54"/>
     </row>
     <row r="13" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A13" s="48" t="s">
+      <c r="A13" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="39"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39"/>
-      <c r="J13" s="40"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="70"/>
+      <c r="H13" s="70"/>
+      <c r="I13" s="70"/>
+      <c r="J13" s="73"/>
     </row>
     <row r="14" spans="1:10" ht="12.75" customHeight="1"/>
     <row r="15" spans="1:10" ht="12.75" customHeight="1"/>
@@ -3997,17 +4026,14 @@
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="D2:E4"/>
-    <mergeCell ref="F2:G4"/>
-    <mergeCell ref="H2:H4"/>
-    <mergeCell ref="I2:I4"/>
-    <mergeCell ref="J2:J4"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:J12"/>
+    <mergeCell ref="D13:J13"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="D7:J7"/>
+    <mergeCell ref="D8:J8"/>
+    <mergeCell ref="D9:J9"/>
+    <mergeCell ref="D10:J10"/>
+    <mergeCell ref="D11:J11"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C4"/>
     <mergeCell ref="A5:C5"/>
@@ -4016,14 +4042,17 @@
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D13:J13"/>
-    <mergeCell ref="D5:J5"/>
-    <mergeCell ref="D6:J6"/>
-    <mergeCell ref="D7:J7"/>
-    <mergeCell ref="D8:J8"/>
-    <mergeCell ref="D9:J9"/>
-    <mergeCell ref="D10:J10"/>
-    <mergeCell ref="D11:J11"/>
+    <mergeCell ref="I2:I4"/>
+    <mergeCell ref="J2:J4"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:J12"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="D2:E4"/>
+    <mergeCell ref="F2:G4"/>
+    <mergeCell ref="H2:H4"/>
   </mergeCells>
   <phoneticPr fontId="8"/>
   <pageMargins left="0.70833333333333304" right="0.70833333333333304" top="0.74791666666666701" bottom="0.74791666666666701" header="0" footer="0"/>
@@ -4042,19 +4071,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="73" t="s">
+      <c r="B1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="73" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="60"/>
+      <c r="G1" s="67"/>
       <c r="H1" s="4" t="s">
         <v>8</v>
       </c>
@@ -4066,40 +4095,40 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="70"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="45"/>
     </row>
     <row r="3" spans="1:10" ht="18" customHeight="1">
-      <c r="A3" s="53"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="71"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="18" customHeight="1">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="77"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
-      <c r="J4" s="72"/>
+      <c r="A4" s="87"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="80"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="82"/>
     </row>
     <row r="5" spans="1:10" ht="12.75" customHeight="1">
       <c r="A5" s="8"/>
@@ -5455,19 +5484,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="73" t="s">
+      <c r="B1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="73" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="60"/>
+      <c r="G1" s="67"/>
       <c r="H1" s="4" t="s">
         <v>8</v>
       </c>
@@ -5479,40 +5508,40 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="70"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="45"/>
     </row>
     <row r="3" spans="1:10" ht="18" customHeight="1">
-      <c r="A3" s="53"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="71"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="18" customHeight="1">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="77"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
-      <c r="J4" s="72"/>
+      <c r="A4" s="87"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="80"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="82"/>
     </row>
     <row r="5" spans="1:10" ht="12.75" customHeight="1">
       <c r="A5" s="8"/>
@@ -6862,19 +6891,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="73" t="s">
+      <c r="B1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="60"/>
-      <c r="F1" s="73" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="60"/>
+      <c r="G1" s="67"/>
       <c r="H1" s="4" t="s">
         <v>8</v>
       </c>
@@ -6886,189 +6915,189 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="70"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="45"/>
     </row>
     <row r="3" spans="1:10" ht="18" customHeight="1">
-      <c r="A3" s="53"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="71"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="46"/>
     </row>
     <row r="4" spans="1:10" ht="18" customHeight="1">
-      <c r="A4" s="53"/>
-      <c r="B4" s="54"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="71"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
+      <c r="J4" s="46"/>
     </row>
     <row r="5" spans="1:10" ht="28.5" customHeight="1">
-      <c r="A5" s="86" t="s">
+      <c r="A5" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="60"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="43"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
     </row>
     <row r="6" spans="1:10" ht="21" customHeight="1">
-      <c r="A6" s="88" t="s">
+      <c r="A6" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="46"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="54"/>
     </row>
     <row r="7" spans="1:10" ht="21" customHeight="1">
-      <c r="A7" s="90"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="92"/>
+      <c r="A7" s="55"/>
+      <c r="B7" s="56"/>
+      <c r="C7" s="56"/>
+      <c r="D7" s="56"/>
+      <c r="E7" s="56"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="56"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="56"/>
+      <c r="J7" s="57"/>
     </row>
     <row r="8" spans="1:10" ht="21" customHeight="1">
-      <c r="A8" s="53"/>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="93"/>
+      <c r="A8" s="58"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="60"/>
     </row>
     <row r="9" spans="1:10" ht="21" customHeight="1">
-      <c r="A9" s="53"/>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
-      <c r="J9" s="93"/>
+      <c r="A9" s="58"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="60"/>
     </row>
     <row r="10" spans="1:10" ht="21" customHeight="1">
-      <c r="A10" s="53"/>
-      <c r="B10" s="54"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
-      <c r="J10" s="93"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="59"/>
+      <c r="J10" s="60"/>
     </row>
     <row r="11" spans="1:10" ht="21" customHeight="1">
-      <c r="A11" s="53"/>
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="54"/>
-      <c r="J11" s="93"/>
+      <c r="A11" s="58"/>
+      <c r="B11" s="59"/>
+      <c r="C11" s="59"/>
+      <c r="D11" s="59"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="60"/>
     </row>
     <row r="12" spans="1:10" ht="21" customHeight="1">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
-      <c r="H12" s="54"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="93"/>
+      <c r="A12" s="58"/>
+      <c r="B12" s="59"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="60"/>
     </row>
     <row r="13" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A13" s="53"/>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="93"/>
+      <c r="A13" s="58"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="59"/>
+      <c r="I13" s="59"/>
+      <c r="J13" s="60"/>
     </row>
     <row r="14" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A14" s="88" t="s">
+      <c r="A14" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="46"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="54"/>
     </row>
     <row r="15" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A15" s="88" t="s">
+      <c r="A15" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="62"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="62"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="49"/>
       <c r="I15" s="15" t="s">
         <v>28</v>
       </c>
       <c r="J15" s="16"/>
     </row>
     <row r="16" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A16" s="88" t="s">
+      <c r="A16" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="45"/>
-      <c r="C16" s="62"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="49"/>
       <c r="D16" s="15" t="s">
         <v>30</v>
       </c>
@@ -7081,95 +7110,95 @@
       <c r="G16" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="94" t="s">
+      <c r="H16" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="45"/>
-      <c r="J16" s="46"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="54"/>
     </row>
     <row r="17" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A17" s="85"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="62"/>
+      <c r="A17" s="50"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="49"/>
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="46"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="54"/>
     </row>
     <row r="18" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A18" s="85"/>
-      <c r="B18" s="45"/>
-      <c r="C18" s="62"/>
+      <c r="A18" s="50"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="49"/>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
       <c r="F18" s="18"/>
       <c r="G18" s="18"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="46"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="54"/>
     </row>
     <row r="19" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A19" s="85"/>
-      <c r="B19" s="45"/>
-      <c r="C19" s="62"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="49"/>
       <c r="D19" s="17"/>
       <c r="E19" s="17"/>
       <c r="F19" s="18"/>
       <c r="G19" s="18"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="46"/>
+      <c r="H19" s="61"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="54"/>
     </row>
     <row r="20" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A20" s="85"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="62"/>
+      <c r="A20" s="50"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="49"/>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
       <c r="F20" s="18"/>
       <c r="G20" s="18"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="46"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="54"/>
     </row>
     <row r="21" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A21" s="85"/>
-      <c r="B21" s="45"/>
-      <c r="C21" s="62"/>
+      <c r="A21" s="50"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="49"/>
       <c r="D21" s="17"/>
       <c r="E21" s="17"/>
       <c r="F21" s="18"/>
       <c r="G21" s="18"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="46"/>
+      <c r="H21" s="61"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="54"/>
     </row>
     <row r="22" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A22" s="85"/>
-      <c r="B22" s="45"/>
-      <c r="C22" s="62"/>
+      <c r="A22" s="50"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="49"/>
       <c r="D22" s="17"/>
       <c r="E22" s="17"/>
       <c r="F22" s="18"/>
       <c r="G22" s="18"/>
-      <c r="H22" s="44"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="46"/>
+      <c r="H22" s="61"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="54"/>
     </row>
     <row r="23" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A23" s="87"/>
-      <c r="B23" s="39"/>
-      <c r="C23" s="49"/>
+      <c r="A23" s="69"/>
+      <c r="B23" s="70"/>
+      <c r="C23" s="71"/>
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
       <c r="F23" s="20"/>
       <c r="G23" s="20"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="40"/>
+      <c r="H23" s="72"/>
+      <c r="I23" s="70"/>
+      <c r="J23" s="73"/>
     </row>
     <row r="24" spans="1:10" ht="12.75" customHeight="1"/>
     <row r="25" spans="1:10" ht="12.75" customHeight="1"/>
@@ -8150,10 +8179,17 @@
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="F2:G4"/>
-    <mergeCell ref="H2:H4"/>
-    <mergeCell ref="I2:I4"/>
-    <mergeCell ref="J2:J4"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="H21:J21"/>
+    <mergeCell ref="H22:J22"/>
     <mergeCell ref="A1:C4"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="D1:E1"/>
@@ -8170,17 +8206,10 @@
     <mergeCell ref="H16:J16"/>
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="D2:E4"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="H21:J21"/>
-    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="F2:G4"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="I2:I4"/>
+    <mergeCell ref="J2:J4"/>
   </mergeCells>
   <phoneticPr fontId="8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -8199,182 +8228,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="18" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="73" t="s">
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="73" t="s">
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="73" t="s">
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="73" t="s">
+      <c r="P1" s="67"/>
+      <c r="Q1" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="R1" s="60"/>
-      <c r="S1" s="73" t="s">
+      <c r="R1" s="67"/>
+      <c r="S1" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="43"/>
+      <c r="T1" s="53"/>
     </row>
     <row r="2" spans="1:26" ht="18" customHeight="1">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="74"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="74"/>
-      <c r="P2" s="75"/>
-      <c r="Q2" s="74"/>
-      <c r="R2" s="75"/>
-      <c r="S2" s="74"/>
-      <c r="T2" s="92"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="39"/>
+      <c r="Q2" s="38"/>
+      <c r="R2" s="39"/>
+      <c r="S2" s="38"/>
+      <c r="T2" s="57"/>
     </row>
     <row r="3" spans="1:26" ht="18" customHeight="1">
-      <c r="A3" s="53"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="76"/>
-      <c r="L3" s="54"/>
-      <c r="M3" s="54"/>
-      <c r="N3" s="55"/>
-      <c r="O3" s="76"/>
-      <c r="P3" s="55"/>
-      <c r="Q3" s="76"/>
-      <c r="R3" s="55"/>
-      <c r="S3" s="76"/>
-      <c r="T3" s="93"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="41"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="41"/>
+      <c r="S3" s="40"/>
+      <c r="T3" s="60"/>
     </row>
     <row r="4" spans="1:26" ht="18" customHeight="1">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="77"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="58"/>
-      <c r="O4" s="77"/>
-      <c r="P4" s="58"/>
-      <c r="Q4" s="77"/>
-      <c r="R4" s="58"/>
-      <c r="S4" s="77"/>
-      <c r="T4" s="103"/>
+      <c r="A4" s="87"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="88"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="80"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="88"/>
+      <c r="M4" s="88"/>
+      <c r="N4" s="80"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="80"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="80"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="98"/>
     </row>
     <row r="5" spans="1:26" ht="18" customHeight="1">
-      <c r="A5" s="86" t="s">
+      <c r="A5" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="41" t="s">
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="67"/>
+      <c r="G5" s="93" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
-      <c r="L5" s="42"/>
-      <c r="M5" s="42"/>
-      <c r="N5" s="42"/>
-      <c r="O5" s="42"/>
-      <c r="P5" s="42"/>
-      <c r="Q5" s="42"/>
-      <c r="R5" s="42"/>
-      <c r="S5" s="42"/>
-      <c r="T5" s="43"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="52"/>
+      <c r="K5" s="52"/>
+      <c r="L5" s="52"/>
+      <c r="M5" s="52"/>
+      <c r="N5" s="52"/>
+      <c r="O5" s="52"/>
+      <c r="P5" s="52"/>
+      <c r="Q5" s="52"/>
+      <c r="R5" s="52"/>
+      <c r="S5" s="52"/>
+      <c r="T5" s="53"/>
     </row>
     <row r="6" spans="1:26" ht="18" customHeight="1">
-      <c r="A6" s="88" t="s">
+      <c r="A6" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="44" t="s">
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
-      <c r="N6" s="45"/>
-      <c r="O6" s="45"/>
-      <c r="P6" s="45"/>
-      <c r="Q6" s="45"/>
-      <c r="R6" s="45"/>
-      <c r="S6" s="45"/>
-      <c r="T6" s="46"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
+      <c r="P6" s="48"/>
+      <c r="Q6" s="48"/>
+      <c r="R6" s="48"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="54"/>
     </row>
     <row r="7" spans="1:26" ht="18" customHeight="1">
-      <c r="A7" s="88" t="s">
+      <c r="A7" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="62"/>
-      <c r="G7" s="44" t="s">
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
-      <c r="O7" s="45"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="46"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="48"/>
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="48"/>
+      <c r="R7" s="48"/>
+      <c r="S7" s="48"/>
+      <c r="T7" s="54"/>
     </row>
     <row r="8" spans="1:26" ht="7.5" customHeight="1">
       <c r="A8" s="8"/>
@@ -8573,37 +8602,37 @@
       <c r="T14" s="10"/>
     </row>
     <row r="15" spans="1:26" ht="18.75" customHeight="1">
-      <c r="A15" s="88" t="s">
+      <c r="A15" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="62"/>
-      <c r="C15" s="102" t="s">
+      <c r="B15" s="49"/>
+      <c r="C15" s="101" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="62"/>
-      <c r="E15" s="94" t="s">
+      <c r="D15" s="49"/>
+      <c r="E15" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="62"/>
-      <c r="G15" s="94" t="s">
+      <c r="F15" s="49"/>
+      <c r="G15" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="H15" s="45"/>
-      <c r="I15" s="62"/>
-      <c r="J15" s="94" t="s">
+      <c r="H15" s="48"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="K15" s="62"/>
-      <c r="L15" s="94" t="s">
+      <c r="K15" s="49"/>
+      <c r="L15" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="M15" s="45"/>
-      <c r="N15" s="62"/>
-      <c r="O15" s="94" t="s">
+      <c r="M15" s="48"/>
+      <c r="N15" s="49"/>
+      <c r="O15" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="P15" s="45"/>
-      <c r="Q15" s="62"/>
+      <c r="P15" s="48"/>
+      <c r="Q15" s="49"/>
       <c r="R15" s="15" t="s">
         <v>52</v>
       </c>
@@ -8615,37 +8644,37 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="48" customHeight="1">
-      <c r="A16" s="95">
+      <c r="A16" s="99">
         <v>1</v>
       </c>
-      <c r="B16" s="62"/>
-      <c r="C16" s="96" t="s">
+      <c r="B16" s="49"/>
+      <c r="C16" s="100" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="62"/>
-      <c r="E16" s="96" t="s">
+      <c r="D16" s="49"/>
+      <c r="E16" s="100" t="s">
         <v>56</v>
       </c>
-      <c r="F16" s="62"/>
-      <c r="G16" s="101" t="s">
+      <c r="F16" s="49"/>
+      <c r="G16" s="94" t="s">
         <v>57</v>
       </c>
-      <c r="H16" s="45"/>
-      <c r="I16" s="62"/>
-      <c r="J16" s="101" t="s">
+      <c r="H16" s="48"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="94" t="s">
         <v>58</v>
       </c>
-      <c r="K16" s="62"/>
-      <c r="L16" s="99" t="s">
+      <c r="K16" s="49"/>
+      <c r="L16" s="96" t="s">
         <v>59</v>
       </c>
-      <c r="M16" s="45"/>
-      <c r="N16" s="62"/>
-      <c r="O16" s="99" t="s">
+      <c r="M16" s="48"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="96" t="s">
         <v>60</v>
       </c>
-      <c r="P16" s="45"/>
-      <c r="Q16" s="62"/>
+      <c r="P16" s="48"/>
+      <c r="Q16" s="49"/>
       <c r="R16" s="33"/>
       <c r="S16" s="33"/>
       <c r="T16" s="34"/>
@@ -8657,37 +8686,37 @@
       <c r="Z16" s="35"/>
     </row>
     <row r="17" spans="1:26" ht="41.25" customHeight="1">
-      <c r="A17" s="95">
+      <c r="A17" s="99">
         <v>2</v>
       </c>
-      <c r="B17" s="62"/>
-      <c r="C17" s="96" t="s">
+      <c r="B17" s="49"/>
+      <c r="C17" s="100" t="s">
         <v>61</v>
       </c>
-      <c r="D17" s="62"/>
-      <c r="E17" s="96" t="s">
+      <c r="D17" s="49"/>
+      <c r="E17" s="100" t="s">
         <v>62</v>
       </c>
-      <c r="F17" s="62"/>
-      <c r="G17" s="101" t="s">
+      <c r="F17" s="49"/>
+      <c r="G17" s="94" t="s">
         <v>63</v>
       </c>
-      <c r="H17" s="45"/>
-      <c r="I17" s="62"/>
-      <c r="J17" s="101" t="s">
+      <c r="H17" s="48"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="94" t="s">
         <v>64</v>
       </c>
-      <c r="K17" s="62"/>
-      <c r="L17" s="99" t="s">
+      <c r="K17" s="49"/>
+      <c r="L17" s="96" t="s">
         <v>65</v>
       </c>
-      <c r="M17" s="45"/>
-      <c r="N17" s="62"/>
-      <c r="O17" s="99" t="s">
+      <c r="M17" s="48"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="96" t="s">
         <v>66</v>
       </c>
-      <c r="P17" s="45"/>
-      <c r="Q17" s="62"/>
+      <c r="P17" s="48"/>
+      <c r="Q17" s="49"/>
       <c r="R17" s="33"/>
       <c r="S17" s="33"/>
       <c r="T17" s="34"/>
@@ -8699,23 +8728,23 @@
       <c r="Z17" s="35"/>
     </row>
     <row r="18" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A18" s="95"/>
-      <c r="B18" s="62"/>
-      <c r="C18" s="96"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="96"/>
-      <c r="F18" s="62"/>
-      <c r="G18" s="101"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="62"/>
-      <c r="J18" s="101"/>
-      <c r="K18" s="62"/>
-      <c r="L18" s="99"/>
-      <c r="M18" s="45"/>
-      <c r="N18" s="62"/>
-      <c r="O18" s="99"/>
-      <c r="P18" s="45"/>
-      <c r="Q18" s="62"/>
+      <c r="A18" s="99"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="100"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="94"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="94"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="96"/>
+      <c r="M18" s="48"/>
+      <c r="N18" s="49"/>
+      <c r="O18" s="96"/>
+      <c r="P18" s="48"/>
+      <c r="Q18" s="49"/>
       <c r="R18" s="33"/>
       <c r="S18" s="33"/>
       <c r="T18" s="34"/>
@@ -8727,23 +8756,23 @@
       <c r="Z18" s="35"/>
     </row>
     <row r="19" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A19" s="95"/>
-      <c r="B19" s="62"/>
-      <c r="C19" s="96"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="96"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="101"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="101"/>
-      <c r="K19" s="62"/>
-      <c r="L19" s="99"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="62"/>
-      <c r="O19" s="99"/>
-      <c r="P19" s="45"/>
-      <c r="Q19" s="62"/>
+      <c r="A19" s="99"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="100"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="100"/>
+      <c r="F19" s="49"/>
+      <c r="G19" s="94"/>
+      <c r="H19" s="48"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="94"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="96"/>
+      <c r="M19" s="48"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="96"/>
+      <c r="P19" s="48"/>
+      <c r="Q19" s="49"/>
       <c r="R19" s="33"/>
       <c r="S19" s="33"/>
       <c r="T19" s="34"/>
@@ -8755,23 +8784,23 @@
       <c r="Z19" s="35"/>
     </row>
     <row r="20" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A20" s="95"/>
-      <c r="B20" s="62"/>
-      <c r="C20" s="96"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="96"/>
-      <c r="F20" s="62"/>
-      <c r="G20" s="101"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="62"/>
-      <c r="J20" s="101"/>
-      <c r="K20" s="62"/>
-      <c r="L20" s="99"/>
-      <c r="M20" s="45"/>
-      <c r="N20" s="62"/>
-      <c r="O20" s="99"/>
-      <c r="P20" s="45"/>
-      <c r="Q20" s="62"/>
+      <c r="A20" s="99"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="100"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="100"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="94"/>
+      <c r="H20" s="48"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="94"/>
+      <c r="K20" s="49"/>
+      <c r="L20" s="96"/>
+      <c r="M20" s="48"/>
+      <c r="N20" s="49"/>
+      <c r="O20" s="96"/>
+      <c r="P20" s="48"/>
+      <c r="Q20" s="49"/>
       <c r="R20" s="33"/>
       <c r="S20" s="33"/>
       <c r="T20" s="34"/>
@@ -8783,23 +8812,23 @@
       <c r="Z20" s="35"/>
     </row>
     <row r="21" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A21" s="95"/>
-      <c r="B21" s="62"/>
-      <c r="C21" s="96"/>
-      <c r="D21" s="62"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="62"/>
-      <c r="G21" s="101"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="62"/>
-      <c r="J21" s="101"/>
-      <c r="K21" s="62"/>
-      <c r="L21" s="99"/>
-      <c r="M21" s="45"/>
-      <c r="N21" s="62"/>
-      <c r="O21" s="99"/>
-      <c r="P21" s="45"/>
-      <c r="Q21" s="62"/>
+      <c r="A21" s="99"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="100"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="100"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="94"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="94"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="96"/>
+      <c r="M21" s="48"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="96"/>
+      <c r="P21" s="48"/>
+      <c r="Q21" s="49"/>
       <c r="R21" s="33"/>
       <c r="S21" s="33"/>
       <c r="T21" s="34"/>
@@ -8811,23 +8840,23 @@
       <c r="Z21" s="35"/>
     </row>
     <row r="22" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A22" s="95"/>
-      <c r="B22" s="62"/>
-      <c r="C22" s="96"/>
-      <c r="D22" s="62"/>
-      <c r="E22" s="96"/>
-      <c r="F22" s="62"/>
-      <c r="G22" s="101"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="62"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="62"/>
-      <c r="L22" s="99"/>
-      <c r="M22" s="45"/>
-      <c r="N22" s="62"/>
-      <c r="O22" s="99"/>
-      <c r="P22" s="45"/>
-      <c r="Q22" s="62"/>
+      <c r="A22" s="99"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="100"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="100"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="94"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="94"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="96"/>
+      <c r="M22" s="48"/>
+      <c r="N22" s="49"/>
+      <c r="O22" s="96"/>
+      <c r="P22" s="48"/>
+      <c r="Q22" s="49"/>
       <c r="R22" s="33"/>
       <c r="S22" s="33"/>
       <c r="T22" s="34"/>
@@ -8839,23 +8868,23 @@
       <c r="Z22" s="35"/>
     </row>
     <row r="23" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A23" s="95"/>
-      <c r="B23" s="62"/>
-      <c r="C23" s="96"/>
-      <c r="D23" s="62"/>
-      <c r="E23" s="96"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="101"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="62"/>
-      <c r="J23" s="101"/>
-      <c r="K23" s="62"/>
-      <c r="L23" s="99"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="62"/>
-      <c r="O23" s="99"/>
-      <c r="P23" s="45"/>
-      <c r="Q23" s="62"/>
+      <c r="A23" s="99"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="100"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="100"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="94"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="96"/>
+      <c r="M23" s="48"/>
+      <c r="N23" s="49"/>
+      <c r="O23" s="96"/>
+      <c r="P23" s="48"/>
+      <c r="Q23" s="49"/>
       <c r="R23" s="33"/>
       <c r="S23" s="33"/>
       <c r="T23" s="34"/>
@@ -8867,23 +8896,23 @@
       <c r="Z23" s="35"/>
     </row>
     <row r="24" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A24" s="95"/>
-      <c r="B24" s="62"/>
-      <c r="C24" s="96"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="96"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="101"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="62"/>
-      <c r="J24" s="101"/>
-      <c r="K24" s="62"/>
-      <c r="L24" s="99"/>
-      <c r="M24" s="45"/>
-      <c r="N24" s="62"/>
-      <c r="O24" s="99"/>
-      <c r="P24" s="45"/>
-      <c r="Q24" s="62"/>
+      <c r="A24" s="99"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="100"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="100"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="94"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="94"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="96"/>
+      <c r="M24" s="48"/>
+      <c r="N24" s="49"/>
+      <c r="O24" s="96"/>
+      <c r="P24" s="48"/>
+      <c r="Q24" s="49"/>
       <c r="R24" s="33"/>
       <c r="S24" s="33"/>
       <c r="T24" s="34"/>
@@ -8895,23 +8924,23 @@
       <c r="Z24" s="35"/>
     </row>
     <row r="25" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A25" s="95"/>
-      <c r="B25" s="62"/>
-      <c r="C25" s="96"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="96"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="101"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="62"/>
-      <c r="J25" s="101"/>
-      <c r="K25" s="62"/>
-      <c r="L25" s="99"/>
-      <c r="M25" s="45"/>
-      <c r="N25" s="62"/>
-      <c r="O25" s="99"/>
-      <c r="P25" s="45"/>
-      <c r="Q25" s="62"/>
+      <c r="A25" s="99"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="100"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="100"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="94"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="94"/>
+      <c r="K25" s="49"/>
+      <c r="L25" s="96"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="49"/>
+      <c r="O25" s="96"/>
+      <c r="P25" s="48"/>
+      <c r="Q25" s="49"/>
       <c r="R25" s="33"/>
       <c r="S25" s="33"/>
       <c r="T25" s="34"/>
@@ -8923,23 +8952,23 @@
       <c r="Z25" s="35"/>
     </row>
     <row r="26" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A26" s="95"/>
-      <c r="B26" s="62"/>
-      <c r="C26" s="96"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="96"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="101"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="62"/>
-      <c r="J26" s="101"/>
-      <c r="K26" s="62"/>
-      <c r="L26" s="99"/>
-      <c r="M26" s="45"/>
-      <c r="N26" s="62"/>
-      <c r="O26" s="99"/>
-      <c r="P26" s="45"/>
-      <c r="Q26" s="62"/>
+      <c r="A26" s="99"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="100"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="100"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="94"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="94"/>
+      <c r="K26" s="49"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="48"/>
+      <c r="N26" s="49"/>
+      <c r="O26" s="96"/>
+      <c r="P26" s="48"/>
+      <c r="Q26" s="49"/>
       <c r="R26" s="33"/>
       <c r="S26" s="33"/>
       <c r="T26" s="34"/>
@@ -8951,23 +8980,23 @@
       <c r="Z26" s="35"/>
     </row>
     <row r="27" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A27" s="95"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="96"/>
-      <c r="D27" s="62"/>
-      <c r="E27" s="96"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="101"/>
-      <c r="H27" s="45"/>
-      <c r="I27" s="62"/>
-      <c r="J27" s="101"/>
-      <c r="K27" s="62"/>
-      <c r="L27" s="99"/>
-      <c r="M27" s="45"/>
-      <c r="N27" s="62"/>
-      <c r="O27" s="99"/>
-      <c r="P27" s="45"/>
-      <c r="Q27" s="62"/>
+      <c r="A27" s="99"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="100"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="100"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="94"/>
+      <c r="H27" s="48"/>
+      <c r="I27" s="49"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="49"/>
+      <c r="L27" s="96"/>
+      <c r="M27" s="48"/>
+      <c r="N27" s="49"/>
+      <c r="O27" s="96"/>
+      <c r="P27" s="48"/>
+      <c r="Q27" s="49"/>
       <c r="R27" s="33"/>
       <c r="S27" s="33"/>
       <c r="T27" s="34"/>
@@ -8979,23 +9008,23 @@
       <c r="Z27" s="35"/>
     </row>
     <row r="28" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A28" s="95"/>
-      <c r="B28" s="62"/>
-      <c r="C28" s="96"/>
-      <c r="D28" s="62"/>
-      <c r="E28" s="96"/>
-      <c r="F28" s="62"/>
-      <c r="G28" s="101"/>
-      <c r="H28" s="45"/>
-      <c r="I28" s="62"/>
-      <c r="J28" s="101"/>
-      <c r="K28" s="62"/>
-      <c r="L28" s="99"/>
-      <c r="M28" s="45"/>
-      <c r="N28" s="62"/>
-      <c r="O28" s="99"/>
-      <c r="P28" s="45"/>
-      <c r="Q28" s="62"/>
+      <c r="A28" s="99"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="100"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="100"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="94"/>
+      <c r="H28" s="48"/>
+      <c r="I28" s="49"/>
+      <c r="J28" s="94"/>
+      <c r="K28" s="49"/>
+      <c r="L28" s="96"/>
+      <c r="M28" s="48"/>
+      <c r="N28" s="49"/>
+      <c r="O28" s="96"/>
+      <c r="P28" s="48"/>
+      <c r="Q28" s="49"/>
       <c r="R28" s="33"/>
       <c r="S28" s="33"/>
       <c r="T28" s="34"/>
@@ -9007,23 +9036,23 @@
       <c r="Z28" s="35"/>
     </row>
     <row r="29" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A29" s="95"/>
-      <c r="B29" s="62"/>
-      <c r="C29" s="96"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="96"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="101"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="62"/>
-      <c r="J29" s="101"/>
-      <c r="K29" s="62"/>
-      <c r="L29" s="99"/>
-      <c r="M29" s="45"/>
-      <c r="N29" s="62"/>
-      <c r="O29" s="99"/>
-      <c r="P29" s="45"/>
-      <c r="Q29" s="62"/>
+      <c r="A29" s="99"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="100"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="100"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="94"/>
+      <c r="H29" s="48"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="94"/>
+      <c r="K29" s="49"/>
+      <c r="L29" s="96"/>
+      <c r="M29" s="48"/>
+      <c r="N29" s="49"/>
+      <c r="O29" s="96"/>
+      <c r="P29" s="48"/>
+      <c r="Q29" s="49"/>
       <c r="R29" s="33"/>
       <c r="S29" s="33"/>
       <c r="T29" s="34"/>
@@ -9035,23 +9064,23 @@
       <c r="Z29" s="35"/>
     </row>
     <row r="30" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A30" s="95"/>
-      <c r="B30" s="62"/>
-      <c r="C30" s="96"/>
-      <c r="D30" s="62"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="62"/>
-      <c r="G30" s="101"/>
-      <c r="H30" s="45"/>
-      <c r="I30" s="62"/>
-      <c r="J30" s="101"/>
-      <c r="K30" s="62"/>
-      <c r="L30" s="99"/>
-      <c r="M30" s="45"/>
-      <c r="N30" s="62"/>
-      <c r="O30" s="99"/>
-      <c r="P30" s="45"/>
-      <c r="Q30" s="62"/>
+      <c r="A30" s="99"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="100"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="100"/>
+      <c r="F30" s="49"/>
+      <c r="G30" s="94"/>
+      <c r="H30" s="48"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="94"/>
+      <c r="K30" s="49"/>
+      <c r="L30" s="96"/>
+      <c r="M30" s="48"/>
+      <c r="N30" s="49"/>
+      <c r="O30" s="96"/>
+      <c r="P30" s="48"/>
+      <c r="Q30" s="49"/>
       <c r="R30" s="33"/>
       <c r="S30" s="33"/>
       <c r="T30" s="34"/>
@@ -9063,23 +9092,23 @@
       <c r="Z30" s="35"/>
     </row>
     <row r="31" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A31" s="97"/>
-      <c r="B31" s="49"/>
-      <c r="C31" s="98"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="98"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="104"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="49"/>
-      <c r="J31" s="104"/>
-      <c r="K31" s="49"/>
-      <c r="L31" s="100"/>
-      <c r="M31" s="39"/>
-      <c r="N31" s="49"/>
-      <c r="O31" s="100"/>
-      <c r="P31" s="39"/>
-      <c r="Q31" s="49"/>
+      <c r="A31" s="102"/>
+      <c r="B31" s="71"/>
+      <c r="C31" s="103"/>
+      <c r="D31" s="71"/>
+      <c r="E31" s="103"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="95"/>
+      <c r="H31" s="70"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="95"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="97"/>
+      <c r="M31" s="70"/>
+      <c r="N31" s="71"/>
+      <c r="O31" s="97"/>
+      <c r="P31" s="70"/>
+      <c r="Q31" s="71"/>
       <c r="R31" s="36"/>
       <c r="S31" s="36"/>
       <c r="T31" s="37"/>
@@ -10077,62 +10106,62 @@
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="136">
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="L26:N26"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="L28:N28"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="L18:N18"/>
-    <mergeCell ref="L19:N19"/>
-    <mergeCell ref="L21:N21"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="L23:N23"/>
-    <mergeCell ref="L24:N24"/>
-    <mergeCell ref="L25:N25"/>
-    <mergeCell ref="K2:N4"/>
-    <mergeCell ref="O2:P4"/>
-    <mergeCell ref="Q2:R4"/>
-    <mergeCell ref="S2:T4"/>
-    <mergeCell ref="A1:F4"/>
-    <mergeCell ref="G1:J1"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="Q1:R1"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="G2:J4"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="O19:Q19"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="O24:Q24"/>
+    <mergeCell ref="O25:Q25"/>
+    <mergeCell ref="O26:Q26"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="G5:T5"/>
     <mergeCell ref="A6:F6"/>
@@ -10157,62 +10186,62 @@
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="O21:Q21"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="O24:Q24"/>
-    <mergeCell ref="O25:Q25"/>
-    <mergeCell ref="O26:Q26"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="K2:N4"/>
+    <mergeCell ref="O2:P4"/>
+    <mergeCell ref="Q2:R4"/>
+    <mergeCell ref="S2:T4"/>
+    <mergeCell ref="A1:F4"/>
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="G2:J4"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="L28:N28"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="L19:N19"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="L25:N25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:K19"/>
   </mergeCells>
   <phoneticPr fontId="8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>